<commit_message>
Remove ExportController and migrate export handling to DocumentService and relevant controllers
</commit_message>
<xml_diff>
--- a/src/main/resources/jxls/template/supply/invoice.xlsx
+++ b/src/main/resources/jxls/template/supply/invoice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nebula\Work\jarkyn-backend\src\main\resources\jxls\template\supply\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBE80053-852B-4168-ABE1-6A71DA9474AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC81741D-F563-4887-85D1-CCF2C2E08D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,10 +141,10 @@
     <t>$[ROW() - ROW(A4)]</t>
   </si>
   <si>
-    <t>Заказ № ${document.name}</t>
-  </si>
-  <si>
     <t>Покупать:</t>
+  </si>
+  <si>
+    <t>Инвойс № ${document.name}</t>
   </si>
 </sst>
 </file>
@@ -776,7 +776,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -786,7 +786,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="16" t="s">

</xml_diff>